<commit_message>
feat(spec): release v3.2.0 baseline with Lemon Squeezy MoR, guest intake, offline recovery key, and 424h WBS
</commit_message>
<xml_diff>
--- a/Resources/WBS.xlsx
+++ b/Resources/WBS.xlsx
@@ -694,7 +694,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>352 Total Hours (264h Academic Baseline + 88h Commercial Extension)</t>
+          <t>424 Total Hours (264h Academic Baseline + 160h Commercial Launch across 18 Weeks)</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Commercial Baseline &amp; Academic Evaluation Specification (Version 3.1.0)</t>
+          <t>Commercial Baseline &amp; Academic Evaluation Specification (Version 3.2.0)</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -856,12 +856,12 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>PostgreSQL Schema &amp; Row-Level Security</t>
+          <t>PostgreSQL Schema, Neon RLS &amp; Hash-Chained Audit</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>Prisma relational schema, PostgreSQL RLS tenant context, and append-only audit grants</t>
+          <t>Prisma relational schema, PostgreSQL RLS tenant context, and append-only audit ledger with SHA-256 prev_hash</t>
         </is>
       </c>
       <c r="F3" s="11" t="inlineStr">
@@ -1056,12 +1056,12 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Email / Password Auth &amp; JWT Sessions</t>
+          <t>Email / Password Auth &amp; Database-Backed Sessions</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Bcrypt password hashing (rounds = 12) and signed HTTP-only JWT cookies</t>
+          <t>Bcrypt/Argon2 password hashing, database-persisted session tokens, and secure HTTP-only cookies</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Token-Bucket Rate Limiter &amp; Pool RLS</t>
+          <t>Shared Store Rate Limiter &amp; Turnstile CAPTCHA</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Token-bucket rate limiting (5 req/hr/IP) on intake + dynamic tenant RLS</t>
+          <t>Shared store rate limiting (Postgres/Upstash) and Turnstile CAPTCHA (5 req/hr/IP)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -1356,12 +1356,12 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>WebCrypto Keypair Generator &amp; KeyStore</t>
+          <t>WebCrypto Keypair Generator &amp; Argon2 S2K KeyStore</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Ed25519 signing + X25519/RSA encryption subkeys in encrypted IndexedDB</t>
+          <t>Ed25519 signing + X25519 encryption keys stored in IndexedDB protected by OpenPGP Argon2 S2K</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Dual-Recipient OpenPGP Payload Encrypt</t>
+          <t>Multi-Recipient OpenPGP Payload Encrypt</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>In-browser payload encryption targeting Org encryption subkey + Hunter key with neutral operational labels</t>
+          <t>In-browser payload encryption targeting Org defenders + Hunter key with neutral operational labels</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>FR-3.4</t>
+          <t>FR-3.5</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -1456,12 +1456,12 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Encrypted Attachment Upload (Cloudflare R2)</t>
+          <t>Direct-to-R2 Presigned Attachment Upload</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Client-side encrypted streaming binary uploads (≤ 25 MB) to R2</t>
+          <t>Client-side encrypted streaming binary uploads (≤ 25 MB) directly to Cloudflare R2 via presigned URLs</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Pure TypeScript CVSS 3.1 &amp; 52-Vector Test</t>
+          <t>Pure TypeScript CVSS 3.1 &amp; 45-Vector Test</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -1706,12 +1706,12 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>GitHub REST API Commit SHA &amp; Author Check</t>
+          <t>GitHub REST API Commit SHA &amp; Branch Check</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>GitHub API v3 lookup validating commit existence, author, and branch for public and private repos</t>
+          <t>GitHub API v3 lookup validating commit existence and branch compare inclusion across public/private repos</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -1991,7 +1991,7 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>WP-BUF</t>
+          <t>WP-BUF-1</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -2056,12 +2056,12 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Auth Hardening &amp; Session Revocation</t>
+          <t>Auth Hardening, TOTP MFA &amp; Password Reset</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>TOTP MFA enrollment, password reset with immediate session revocation (JWT jti blacklisting), and MFA recovery codes</t>
+          <t>TOTP MFA enrollment, password reset with immediate session revocation, encrypted totp_secret at rest</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
@@ -2070,7 +2070,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
@@ -2106,12 +2106,12 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Guided Onboarding &amp; Domain Verification</t>
+          <t>Guided Onboarding &amp; Offline Org Recovery Key</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>Step-by-step wizard: DNS TXT verification, PGP key generation, RFC 9116 download, and public program activation</t>
+          <t>Step-by-step wizard: DNS verification, Offline Master Recovery Key generation, mandatory backup test challenge</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
@@ -2120,7 +2120,7 @@
         </is>
       </c>
       <c r="G28" s="9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>FR-1.5</t>
+          <t>FR-1.6</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -2156,12 +2156,12 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Private Program Access &amp; Invite Lifecycle</t>
+          <t>Account-Less Guest Submission &amp; Tracking URLs</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Cryptographic invitation tokens (`token_hash` SHA-256 storage, 72h expiry, one-time redemption, uninvited email rejection)</t>
+          <t>Ephemeral Curve25519 key generation in browser, secret tracking URL issuance (`/report/track/BBT-RPT-XXXX`), anonymous retests</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="G29" s="11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>WP-2.1</t>
+          <t>WP-4.1</t>
         </is>
       </c>
       <c r="J29" s="11" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>FR-3.6</t>
+          <t>FR-8.4</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -2206,17 +2206,17 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Multi-Defender Keying &amp; Session Re-Wrapping</t>
+          <t>Direct-to-R2 Presigned Upload &amp; Orphan Cleanup</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>Local key export UI, program keyring versioning (`recipient_set_version`), and audited historical session-key re-wrapping</t>
+          <t>Presigned S3/R2 direct upload route (`/api/uploads/presign`), upload quota verification at issuance, and automated orphan cleanup</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>W15–W16</t>
+          <t>W13–W14</t>
         </is>
       </c>
       <c r="G30" s="9" t="n">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="I30" s="9" t="inlineStr">
         <is>
-          <t>WP-3.4</t>
+          <t>WP-4.2</t>
         </is>
       </c>
       <c r="J30" s="9" t="inlineStr">
@@ -2256,12 +2256,12 @@
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Notification Outbox Worker &amp; Deduplication</t>
+          <t>SLA Countdown Engine &amp; Slack Webhooks</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Outbox table pattern, exponential backoff retries, idempotency keys (no duplicate alerts), and minimal-metadata email templates</t>
+          <t>Hourly scheduled SLA cron check, notification outbox worker, visual countdown alerts, and Slack-compatible webhook payloads</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
@@ -2270,7 +2270,7 @@
         </is>
       </c>
       <c r="G31" s="11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>FR-7.5</t>
+          <t>FR-7.7</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
@@ -2306,12 +2306,12 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Redacted Evidence Export Engine</t>
+          <t>Redacted Evidence Export Engine (PDF &amp; JSON)</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Browser-side PDF/JSON export after local decryption. Excludes free-text exploit details by default; includes full preview before download</t>
+          <t>Sanitized PDF and JSON closure summary generation documenting timeline, commit SHA/branch, deployment env, and retest attestations</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>FR-8.4</t>
+          <t>FR-8.6</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -2356,17 +2356,17 @@
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>Production Cloud &amp; Stripe Subscriptions</t>
+          <t>Merchant of Record (Lemon Squeezy) Billing</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Stripe Checkout, Customer Portal, webhook idempotency, failed payment grace periods, cancellation downgrade, and seat entitlement checks</t>
+          <t>Lemon Squeezy checkout integration (49/mo Team &amp; Free Tier), webhook handler, subscription downgrade, direct bank payouts to Pakistan</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>W17–W18</t>
+          <t>W15–W16</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>WP-1.1</t>
+          <t>WP-2.1</t>
         </is>
       </c>
       <c r="J33" s="11" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>FR-8.5</t>
+          <t>FR-2.1</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -2406,21 +2406,21 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>Disaster Recovery &amp; Incident Runbooks</t>
+          <t>Landing Page, Public Docs &amp; Legal Pack</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>Automated daily PostgreSQL + R2 backup restore drill in sandbox, customer hard-deletion workflow, and incident response runbook</t>
+          <t>Marketing landing page, public documentation, free RFC 9116 generator tool, Terms of Service, Privacy Policy, DPA, and subprocessor list</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>W17–W18</t>
+          <t>W15–W16</t>
         </is>
       </c>
       <c r="G34" s="9" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>WP-1.2</t>
+          <t>WP-3.1</t>
         </is>
       </c>
       <c r="J34" s="9" t="inlineStr">
@@ -2446,57 +2446,257 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
+          <t>FR-8.1</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Application Security Hardening &amp; Pen-Test Pass</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>Strict CSP, Subresource Integrity (SRI), CSRF protection on cookies, login/MFA lockout, SSRF checks on GitHub URLs, and self pen-test</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>W17–W18</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>WP-1.3</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>WP-7.10</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>NFR-01</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Observability (Sentry), Environments &amp; Uptime</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>Sentry error tracking, staging and production database migrations in CI, and external uptime monitoring (BetterStack/UptimeRobot)</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>W17–W18</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>WP-1.1</t>
+        </is>
+      </c>
+      <c r="J36" s="9" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>WP-7.11</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>FR-1.2</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>SuperAdmin Abuse Management &amp; Console</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>Administrative dashboard to inspect tenant counts, view platform error rates, handle abuse reports, and suspend abusive tenants</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>W13–W14</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>WP-2.3</t>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>WP-7.12</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>FR-8.7</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Disaster Recovery &amp; GDPR Hard Deletion</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>Automated daily PostgreSQL + R2 backup restore drill in sandbox, customer hard-deletion workflow, and incident response runbook</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>W17–W18</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I38" s="9" t="inlineStr">
+        <is>
+          <t>WP-1.2</t>
+        </is>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>WP-BUF-2</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
           <t>GOV-02</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>GOV: Contingency &amp; Buffer</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>Commercial Launch Contingency Buffer</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>Buffer for unexpected billing edge cases, webhook debugging, and production pilot support</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
-        <is>
-          <t>W13–W18</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="H35" s="11" t="inlineStr">
-        <is>
-          <t>Taha Asadullah</t>
-        </is>
-      </c>
-      <c r="I35" s="11" t="inlineStr">
-        <is>
-          <t>WP-7.1</t>
-        </is>
-      </c>
-      <c r="J35" s="11" t="inlineStr">
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>Commercial Pilot Support &amp; Launch Buffer</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>Buffer for unexpected billing edge cases, webhook debugging, and production pilot customer support</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>W17–W18</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>WP-7.7</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
         <is>
           <t>[ROADMAP]</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="E36" s="13" t="inlineStr">
+    <row r="40">
+      <c r="E40" s="13" t="inlineStr">
         <is>
           <t>TOTAL ESTIMATED ENGINEERING HOURS:</t>
         </is>
       </c>
-      <c r="G36" s="14">
-        <f>SUM(G2:G35)</f>
-        <v>352</v>
+      <c r="G40" s="14">
+        <f>SUM(G2:G39)</f>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -2510,7 +2710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2721,7 +2921,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Attested Retest, Peer Study &amp; Defense</t>
+          <t>Attested Retest &amp; Quota Management</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -2741,7 +2941,71 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Advised by Elena (QA) &amp; Alexander (PM)</t>
+          <t>Advised by Elena (QA) &amp; Garrison (SRE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>MOD-7</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Commercial Deployment, Billing &amp; Hardening</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>A / R</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Advised by Garrison (SRE) &amp; Nadia (Release)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>ACAD</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Usability Study &amp; FYP Defense</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>A / R</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Advised by Alexander (Steward) &amp; Victoria (Req)</t>
         </is>
       </c>
     </row>
@@ -2756,7 +3020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2818,21 +3082,21 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>WP-1.1, WP-1.2, WP-1.3, WP-1.4, Buffer (4h)</t>
+          <t>WP-1.1, WP-1.2, WP-1.3, WP-1.4</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Monorepo scaffolding, PostgreSQL RLS schema, AST Markdown sanitization, design tokens, BRD, SRS, WBS</t>
+          <t>Monorepo scaffolding, PostgreSQL RLS schema, AST sanitization, and UI tokens</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>Phase Gate 1 (DoR) Certified</t>
+          <t>Gate 0: Foundation Review</t>
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
@@ -2853,21 +3117,21 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>WP-2.1, WP-2.2, WP-2.3, WP-2.4, Buffer (4h)</t>
+          <t>WP-2.1, WP-2.2, WP-2.3, WP-2.4</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Tenant registration wizard, bcrypt auth, JWT cookies, server RBAC, token-bucket rate limiter</t>
+          <t>Tenant registration, DB-backed sessions, server RBAC, and shared store rate limiter</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>Phase Gate 2 (DoAC) Architecture</t>
+          <t>Gate 1: Identity &amp; Multi-Tenancy</t>
         </is>
       </c>
       <c r="F3" s="11" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
@@ -2888,21 +3152,21 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>WP-3.1, WP-3.2, WP-3.3, WP-3.4, Buffer (4h)</t>
+          <t>WP-3.1, WP-3.2, WP-3.3, WP-3.4</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Dynamic security.txt download API, browser cleartext PGP signing, DNS TXT check, WebCrypto keypairs</t>
+          <t>RFC 9116 download, in-browser PGP cleartext signing, DNS TXT verifier, Ed25519 keypair generator</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>Phase Gate 3 (DoCC) Core Crypto</t>
+          <t>Gate 2: Policy &amp; Keys</t>
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
@@ -2923,21 +3187,21 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>WP-4.1, WP-4.2, WP-4.3, WP-4.4, Buffer (4h)</t>
+          <t>WP-4.1, WP-4.2, WP-4.3, WP-4.4</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Multi-recipient payload encryption, R2 attachment upload, CVSS 3.1 engine, in-browser decryption, basic triage</t>
+          <t>Dual-recipient encryption, direct R2 presigned upload, pure TS CVSS 3.1 engine, in-browser decryption</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Week 7 Live Working Prototype Milestone</t>
+          <t>Gate 3: Working Prototype Demonstration</t>
         </is>
       </c>
       <c r="F5" s="11" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
@@ -2958,21 +3222,21 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>WP-5.1, WP-5.2, WP-5.3, WP-5.4, Buffer (6h)</t>
+          <t>WP-5.1, WP-5.2, WP-5.3, WP-5.4</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Dual-lane triage threads, Resend metadata alerts, duplicate linking, GitHub REST API commit validation</t>
+          <t>Dual-lane triage threads, metadata email alerts, GitHub commit &amp; branch compare validation, config SHA binder</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Phase Gate 4 (DoQV) Triage &amp; VCS</t>
+          <t>Gate 4: Remediation Evidence</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
@@ -2993,21 +3257,21 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>WP-6.1, WP-6.2, ACAD-01, ACAD-02, Buffer (6h)</t>
+          <t>WP-6.1, WP-6.2, ACAD-01, ACAD-02, WP-BUF-1</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Attested retest engine, storage quotas, peer study (3–5 peers), Final FYP Report &amp; Defense</t>
+          <t>Attested retest state machine, storage quotas, Juice Shop usability study, final thesis &amp; demo defense</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Final FYP Defense &amp; Demonstration</t>
+          <t>Gate 5: Academic FYP Defense Certified</t>
         </is>
       </c>
       <c r="F7" s="11" t="n">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
@@ -3023,26 +3287,26 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Weeks 13–15</t>
+          <t>Weeks 13–14</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>WP-7.1, WP-7.2, WP-7.3, WP-7.4, Buffer (4h)</t>
+          <t>WP-7.1, WP-7.2, WP-7.3, WP-7.4, WP-7.11</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>TOTP MFA, session revocation, guided onboarding wizard, tokenized private programs, multi-defender key management</t>
+          <t>TOTP MFA, offline recovery key onboarding, account-less guest intake, direct R2 upload hardening, SuperAdmin</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Milestone 3: Controlled Commercial Pilot</t>
+          <t>Gate 6: Commercial Core Intake</t>
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
@@ -3058,26 +3322,26 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Weeks 16–18</t>
+          <t>Weeks 15–16</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>WP-7.5, WP-7.6, WP-7.7, WP-7.8, Buffer (6h)</t>
+          <t>WP-7.5, WP-7.6, WP-7.7, WP-7.8</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Notification outbox worker, redacted evidence export engine, Stripe subscription lifecycle, DR sandbox restore</t>
+          <t>SLA countdown engine &amp; Slack webhooks, redacted PDF export, Lemon Squeezy MoR billing, landing page &amp; legal</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Milestone 4: Commercial Launch Gate (DoRG)</t>
+          <t>Gate 7: Commercial Operations Ready</t>
         </is>
       </c>
       <c r="F9" s="11" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
@@ -3086,14 +3350,49 @@
       </c>
     </row>
     <row r="10">
-      <c r="E10" s="13" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 9</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Weeks 17–18</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>WP-7.9, WP-7.10, WP-7.12, WP-BUF-2</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Security hardening &amp; pen-test pass, Sentry observability, disaster recovery sandbox drill, launch buffer</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Gate 8: Commercial Production Release</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>TOTAL PLANNED SPRINT HOURS:</t>
         </is>
       </c>
-      <c r="F10" s="14">
-        <f>SUM(F2:F9)</f>
-        <v>352</v>
+      <c r="F11" s="14">
+        <f>SUM(F2:F10)</f>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -3107,7 +3406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3147,7 +3446,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Client Web &amp; API Gateway</t>
+          <t>Application &amp; API Gateway</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
@@ -3157,16 +3456,16 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Hobby / Free Tier</t>
+          <t>Hobby Developer Tier</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Serverless Functions, Edge CDN, Global SSL</t>
+          <t>Edge CDN, serverless functions, global SSL certificate</t>
         </is>
       </c>
       <c r="E2" s="16" t="n">
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="3">
@@ -3177,27 +3476,27 @@
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Neon Serverless Cloud</t>
+          <t>Neon Serverless</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>Free Tier</t>
+          <t>PostgreSQL Free Tier</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>PostgreSQL 16 (512 MB Storage, Shared Compute, Dynamic RLS)</t>
+          <t>512 MB storage, connection pooling via PgBouncer (50 MB / tenant demo)</t>
         </is>
       </c>
       <c r="E3" s="17" t="n">
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Encrypted Object Storage</t>
+          <t>Encrypted File Storage</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -3207,16 +3506,16 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Free Tier</t>
+          <t>Free Tier Object Storage</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>10 GB Storage, Zero Egress Fees</t>
+          <t>10 GB storage allowance, zero egress bandwidth fees (2 GB / tenant demo)</t>
         </is>
       </c>
       <c r="E4" s="16" t="n">
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="5">
@@ -3232,276 +3531,51 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>Free Developer Tier</t>
+          <t>Developer Free Tier</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>100 Emails / Day, 3,000 Emails / Month</t>
+          <t>3,000 minimal-metadata triage notifications / month</t>
         </is>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Source Code &amp; CI/CD</t>
+          <t>CI/CD Build Automation</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>GitHub Free Tier</t>
+          <t>GitHub Actions</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Public Repository</t>
+          <t>Standard Runner Free Tier</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>2,000 Action Minutes / Month, REST API v3 Integration</t>
+          <t>2,000 automated build &amp; test minutes / month</t>
         </is>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>DNS Resolution</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>System DNS Resolver</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>Free Native</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Node.js `dns.promises` Resolver for Domain Validation</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Domain &amp; SSL</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Local / Vercel Subdomain</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Free Tier</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>`.vercel.app` Free Subdomain with Automatic TLS Certificate</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Production Web Hosting</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Vercel Pro</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Custom domain, isolated team compute</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>**$20.00**</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>Production Database</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Neon Serverless Launch</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>10 GB Storage, automated daily backups</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>**$19.00**</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Encrypted Storage (R2)</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Cloudflare R2 Standard</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>50 GB pooled storage baseline</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>**$0.75**</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Transactional Email</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Resend Pro</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>50,000 emails/mo, dedicated domain</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>**$20.00**</t>
-        </is>
-      </c>
-      <c r="E12" s="16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Custom Domain &amp; DNS</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Cloudflare Registrar</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>`.com` / `.security` TLD</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>**$1.25**</t>
-        </is>
-      </c>
-      <c r="E13" s="17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>Payment Gateway</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Stripe Connect / Billing</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Automated subscription invoicing</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>**Variable**</t>
-        </is>
-      </c>
-      <c r="E14" s="16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>TOTAL FIXED INFRASTRUCTURE</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>**Baseline for ~10–25 Active Tenants**</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>**$61.00 / month**</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>TOTAL DEMO INFRASTRUCTURE COST:</t>
         </is>
       </c>
-      <c r="E16" s="18">
-        <f>SUM(E2:E15)</f>
+      <c r="E7" s="18">
+        <f>SUM(E2:E6)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(spec): resolve critical audit findings, synchronize canonical diagrams, enforce task honesty, and expand linter to 101 checks
</commit_message>
<xml_diff>
--- a/Resources/WBS.xlsx
+++ b/Resources/WBS.xlsx
@@ -834,7 +834,7 @@
       </c>
       <c r="J2" s="9" t="inlineStr">
         <is>
-          <t>[DONE]</t>
+          <t>[READY]</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>[DONE]</t>
+          <t>[READY]</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="J4" s="9" t="inlineStr">
         <is>
-          <t>[DONE]</t>
+          <t>[READY]</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>[DONE]</t>
+          <t>[READY]</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="J6" s="9" t="inlineStr">
         <is>
-          <t>[READY]</t>
+          <t>[PLANNED]</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>[DONE]</t>
+          <t>[READY]</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>[READY]</t>
+          <t>[PLANNED]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(docs): purge internal AI agent personas from academic specifications and documentation
</commit_message>
<xml_diff>
--- a/Resources/WBS.xlsx
+++ b/Resources/WBS.xlsx
@@ -2749,7 +2749,7 @@
       </c>
       <c r="F1" s="15" t="inlineStr">
         <is>
-          <t>Internal AI Advisory Squad</t>
+          <t>Technical Standards &amp; Reference</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>Advised by Arthur (Arch) &amp; Cyra (Sec)</t>
+          <t>PostgreSQL Row-Level Security &amp; OWASP ASVS v4.0</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>Advised by Marcus (Forge) &amp; Cyra (Sec)</t>
+          <t>NIST SP 800-63B Authentication &amp; Multi-Tenant RBAC</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>Advised by Victoria (Req) &amp; Cyra (Sec)</t>
+          <t>IETF RFC 9116 (security.txt) &amp; W3C WebCrypto API</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Advised by Cyra (Sec) &amp; Elena (QA)</t>
+          <t>IETF RFC 9580 (OpenPGP v6) &amp; FIRST CVSS 3.1 Standard</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2909,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Advised by Marcus (Forge) &amp; Julian (UX)</t>
+          <t>GitHub REST API v3 &amp; ISO/IEC 29147 Vulnerability Disclosure</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Advised by Elena (QA) &amp; Garrison (SRE)</t>
+          <t>ISO/IEC 30111 Vulnerability Handling Processes</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Advised by Garrison (SRE) &amp; Nadia (Release)</t>
+          <t>SaaS Merchant-of-Record &amp; Cloud Security Hardening</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Advised by Alexander (Steward) &amp; Victoria (Req)</t>
+          <t>IEEE 830-1998 Standards &amp; PTUT FYP Evaluation Criteria</t>
         </is>
       </c>
     </row>

</xml_diff>